<commit_message>
Archive HDLBits Q8 progress
</commit_message>
<xml_diff>
--- a/outputs/hdlbits-archive/HDLBits_Tracker.xlsx
+++ b/outputs/hdlbits-archive/HDLBits_Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rda21839dd2fb4ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R641a44991dc64ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R06f55543237b4f7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R620c29682a984bc1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
     <x:numFmt numFmtId="201" formatCode="0%"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -100,8 +100,13 @@
       <x:color rgb="FF0563C1"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F1F1F"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -136,6 +141,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFF99"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCCFFCC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E1F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -190,7 +210,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="119">
+  <x:cellXfs count="130">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -504,6 +524,17 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="14" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="14" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -514,7 +545,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFCCFFCC"/>
         </x:patternFill>
       </x:fill>
@@ -525,7 +556,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFFF99"/>
         </x:patternFill>
       </x:fill>
@@ -535,7 +566,7 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3F3F3"/>
         </x:patternFill>
       </x:fill>
@@ -545,7 +576,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFCCFFCC"/>
         </x:patternFill>
       </x:fill>
@@ -814,7 +845,7 @@
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="92" t="str">
         <x:f>"Exact website sequence · "&amp;A6&amp;" of "&amp;D6&amp;" completed · "&amp;B6&amp;" review · "&amp;C6&amp;" to do"</x:f>
-        <x:v>Exact website sequence · 140 of 178 completed · 1 review · 37 to do</x:v>
+        <x:v>Exact website sequence · 141 of 178 completed · 2 review · 35 to do</x:v>
       </x:c>
       <x:c r="B3" s="92"/>
       <x:c r="C3" s="92"/>
@@ -850,15 +881,15 @@
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="97" t="n">
         <x:f>COUNTIF('Tracker'!$G$6:$G$260,"Completed")</x:f>
-        <x:v>140</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B6" s="97" t="n">
         <x:f>COUNTIF('Tracker'!$G$6:$G$260,"Review")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="97" t="n">
         <x:f>COUNTIF('Tracker'!$G$6:$G$260,"To Do")</x:f>
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D6" s="97" t="n">
         <x:f>COUNTA('Tracker'!$F$6:$F$260)</x:f>
@@ -868,7 +899,7 @@
         <x:v>Problem</x:v>
       </x:c>
       <x:c r="G6" s="106" t="str">
-        <x:v>Lemmings 2</x:v>
+        <x:v>Lemmings 2; Q2a: FSM</x:v>
       </x:c>
       <x:c r="H6" s="106"/>
     </x:row>
@@ -877,7 +908,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="G7" s="106" t="str">
-        <x:v>Review — 7 unsuccessful attempts</x:v>
+        <x:v>Review - 10 unsuccessful attempts</x:v>
       </x:c>
       <x:c r="H7" s="106"/>
     </x:row>
@@ -892,7 +923,7 @@
         <x:v>Source</x:v>
       </x:c>
       <x:c r="G8" s="107" t="str">
-        <x:v>https://hdlbits.01xz.net/wiki/lemmings2</x:v>
+        <x:v>Review.md</x:v>
       </x:c>
       <x:c r="H8" s="107"/>
     </x:row>
@@ -1076,6 +1107,16 @@
       </x:c>
     </x:row>
     <x:row r="17">
+      <x:c r="A17" s="125" t="str">
+        <x:v>Day 07</x:v>
+      </x:c>
+      <x:c r="B17" s="128" t="n">
+        <x:v>46202</x:v>
+      </x:c>
+      <x:c r="C17" s="129" t="n">
+        <x:f>COUNTIFS('Tracker'!$H$6:$H$260,A17,'Tracker'!$G$6:$G$260,"Completed")</x:f>
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="E17" s="117" t="str">
         <x:v>Circuits</x:v>
       </x:c>
@@ -1212,7 +1253,7 @@
       </x:c>
       <x:c r="G25" s="118" t="n">
         <x:f>COUNTIFS('Tracker'!$C$6:$C$260,E25,'Tracker'!$D$6:$D$260,F25,'Tracker'!$G$6:$G$260,"Completed")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H25" s="118" t="n">
         <x:f>COUNTIFS('Tracker'!$C$6:$C$260,E25,'Tracker'!$D$6:$D$260,F25)</x:f>
@@ -1462,7 +1503,7 @@
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="8" t="str">
         <x:f>"Website sequence verified: 178 of 178 IDs in exact order · "&amp;COUNTIF($G$6:$G$260,"Completed")&amp;" completed · "&amp;COUNTIF($G$6:$G$260,"Review")&amp;" review · "&amp;COUNTIF($G$6:$G$260,"To Do")&amp;" to do"</x:f>
-        <x:v>Website sequence verified: 178 of 178 IDs in exact order · 140 completed · 1 review · 37 to do</x:v>
+        <x:v>Website sequence verified: 178 of 178 IDs in exact order · 141 completed · 2 review · 35 to do</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -10878,7 +10919,9 @@
       <x:c r="A161" s="26" t="n">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="B161" s="26"/>
+      <x:c r="B161" s="26" t="n">
+        <x:v>142</x:v>
+      </x:c>
       <x:c r="C161" s="23" t="str">
         <x:v>Circuits</x:v>
       </x:c>
@@ -10892,33 +10935,50 @@
         <x:v>exams/ece241_2013_q8</x:v>
       </x:c>
       <x:c r="G161" s="26" t="str">
-        <x:v>To Do</x:v>
-      </x:c>
-      <x:c r="H161" s="26"/>
-      <x:c r="I161" s="32"/>
-      <x:c r="J161" s="26"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="H161" s="26" t="str">
+        <x:v>Day 07</x:v>
+      </x:c>
+      <x:c r="I161" s="32" t="n">
+        <x:v>46202</x:v>
+      </x:c>
+      <x:c r="J161" s="26" t="str">
+        <x:v>12:02:40 AM</x:v>
+      </x:c>
       <x:c r="K161" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L161" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M161" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N161" s="26" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O161" s="35"/>
-      <x:c r="P161" s="29"/>
-      <x:c r="Q161" s="29"/>
-      <x:c r="R161" s="29"/>
+      <x:c r="O161" s="35" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="P161" s="29" t="e">
+        <x:f>HYPERLINK("https://github.com/kapiltrip/hdlBits/blob/main/problems/Day%2007/142-exams__ece241_2013_q8.md","Note")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/kapiltrip/hdlBits/blob/main/problems/Day%2007/142-exams__ece241_2013_q8.md, friendlyName=Note</x:v>
+      </x:c>
+      <x:c r="Q161" s="29" t="e">
+        <x:f>HYPERLINK("https://github.com/kapiltrip/hdlBits/blob/main/images/Day%2007/142-exams__ece241_2013_q8.png","Image")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/kapiltrip/hdlBits/blob/main/images/Day%2007/142-exams__ece241_2013_q8.png, friendlyName=Image</x:v>
+      </x:c>
+      <x:c r="R161" s="29" t="e">
+        <x:f>HYPERLINK("https://github.com/kapiltrip/hdlBits/blob/main/solutions/Day%2007/142-exams__ece241_2013_q8.sv","Code")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/kapiltrip/hdlBits/blob/main/solutions/Day%2007/142-exams__ece241_2013_q8.sv, friendlyName=Code</x:v>
+      </x:c>
       <x:c r="S161" s="29" t="e">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/ece241_2013_q8","HDLBits")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://hdlbits.01xz.net/wiki/exams/ece241_2013_q8, friendlyName=HDLBits</x:v>
       </x:c>
       <x:c r="T161" s="23" t="str">
-        <x:v>Not attempted yet. Read the HDLBits question, design the circuit or testbench, and obtain a successful submission.</x:v>
+        <x:v>Three-state Mealy detector for overlapping 101 with active-low asynchronous reset. State S10 plus input 1 asserts z in the detection cycle.</x:v>
       </x:c>
       <x:c r="U161" s="23"/>
     </x:row>
@@ -11420,33 +11480,41 @@
         <x:v>exams/2013_q2afsm</x:v>
       </x:c>
       <x:c r="G172" s="49" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Review</x:v>
       </x:c>
       <x:c r="H172" s="49"/>
       <x:c r="I172" s="51"/>
       <x:c r="J172" s="49"/>
       <x:c r="K172" s="49" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L172" s="49" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M172" s="49" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N172" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="O172" s="52"/>
-      <x:c r="P172" s="53"/>
-      <x:c r="Q172" s="53"/>
+      <x:c r="O172" s="52" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P172" s="53" t="e">
+        <x:f>HYPERLINK("https://github.com/kapiltrip/hdlBits/blob/main/Review.md","Review")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/kapiltrip/hdlBits/blob/main/Review.md, friendlyName=Review</x:v>
+      </x:c>
+      <x:c r="Q172" s="53" t="e">
+        <x:f>HYPERLINK("https://github.com/kapiltrip/hdlBits/blob/main/images/Review/review-exams__2013_q2afsm.png","Image")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/kapiltrip/hdlBits/blob/main/images/Review/review-exams__2013_q2afsm.png, friendlyName=Image</x:v>
+      </x:c>
       <x:c r="R172" s="53"/>
       <x:c r="S172" s="53" t="e">
         <x:f>HYPERLINK("https://hdlbits.01xz.net/wiki/exams/2013_q2afsm","HDLBits")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://hdlbits.01xz.net/wiki/exams/2013_q2afsm, friendlyName=HDLBits</x:v>
       </x:c>
       <x:c r="T172" s="50" t="str">
-        <x:v>Not attempted yet. Read the HDLBits question, design the circuit or testbench, and obtain a successful submission.</x:v>
+        <x:v>Attempted but not yet solved. Review the arbiter state diagram, request priority rules, and grant-hold behavior before resubmitting.</x:v>
       </x:c>
       <x:c r="U172" s="50"/>
     </x:row>

</xml_diff>